<commit_message>
feat: add official HSC 2026 routine notice pages
Add the three-page official HSC 2026 routine notice to the HSC routine guide, with optimized WebP images, bilingual captions, full-size links and a PDF download. Rebuild the generated pages and metadata.
</commit_message>
<xml_diff>
--- a/SEO_Tracker.xlsx
+++ b/SEO_Tracker.xlsx
@@ -1270,7 +1270,7 @@
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/ssc.html</t>
+          <t>https://boardexambd.com/ssc</t>
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/hsc.html</t>
+          <t>https://boardexambd.com/hsc</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/admission.html</t>
+          <t>https://boardexambd.com/admission</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/blog.html</t>
+          <t>https://boardexambd.com/blog</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/ssc-2026-routine.html</t>
+          <t>https://boardexambd.com/ssc-2026-routine</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/ssc-2026-result.html</t>
+          <t>https://boardexambd.com/ssc-2026-result</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/ssc-form-fillup-2027.html</t>
+          <t>https://boardexambd.com/ssc-form-fillup-2027</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/ssc-board-challenge-2026.html</t>
+          <t>https://boardexambd.com/ssc-board-challenge-2026</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/hsc-2026-routine.html</t>
+          <t>https://boardexambd.com/hsc-2026-routine</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/hsc-2026-result.html</t>
+          <t>https://boardexambd.com/hsc-2026-result</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/hsc-form-fillup-2027.html</t>
+          <t>https://boardexambd.com/hsc-form-fillup-2027</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
@@ -2678,7 +2678,7 @@
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/hsc-practical-2026.html</t>
+          <t>https://boardexambd.com/hsc-practical-2026</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/buet-admission-2026-27.html</t>
+          <t>https://boardexambd.com/buet-admission-2026-27</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
@@ -2934,7 +2934,7 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/du-a-unit-admission-2026-27.html</t>
+          <t>https://boardexambd.com/du-a-unit-admission-2026-27</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -3062,7 +3062,7 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/gst-a-unit-admission-2026-27.html</t>
+          <t>https://boardexambd.com/gst-a-unit-admission-2026-27</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/ku-admission-2026-27.html</t>
+          <t>https://boardexambd.com/ku-admission-2026-27</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/medical-admission-2026-27.html</t>
+          <t>https://boardexambd.com/medical-admission-2026-27</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
@@ -3446,7 +3446,7 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/ru-admission-2026-27.html</t>
+          <t>https://boardexambd.com/ru-admission-2026-27</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -3574,7 +3574,7 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/ruet-admission-2026-27.html</t>
+          <t>https://boardexambd.com/ruet-admission-2026-27</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
@@ -3702,7 +3702,7 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/sust-admission-2026-27.html</t>
+          <t>https://boardexambd.com/sust-admission-2026-27</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -3830,7 +3830,7 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>https://boardexambd.com/404.html</t>
+          <t>https://boardexambd.com/404</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Fix HSC result date to 31 Oct 2026 across build sources
The site is fully generated by tools/build_site.py, so the 29 Oct date in
the HTML was being reverted on every rebuild. Fixed the source of truth
instead of the generated output:

- seo_config.py: HSC result description/FAQ to published Saturday
  31 October 2026, SMS number 16222 -> 16140, modified/next_review dates
- hub_renderers.py: hub fact card, HSC timeline and home dates/timeline
  now show 31 Oct 2026 with Published status and correct ISO date
- site_components.py + build_site.py: site-wide updated date to 31 Oct 2026
- HTML body blocks: scheduled -> published, Thursday -> Saturday
- make_tracker.py / README / SEO_IMPLEMENTATION_PLAN: stale 29 Oct refs

Also restored ssc-26-routine/ PNGs, accidentally deleted in 5b62fe3, which
was breaking npm run build at the stage step. Verified byte-identical to
the originals in pdf/ssc-26-routine/.

Build: npm run build -> 21 indexable pages, 22 staged pages, 62 files.
</commit_message>
<xml_diff>
--- a/SEO_Tracker.xlsx
+++ b/SEO_Tracker.xlsx
@@ -22,10 +22,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-  </numFmts>
-  <fonts count="8">
+  <numFmts count="0"/>
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,12 +57,8 @@
       <color rgb="001D4ED8"/>
       <u val="single"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00166534"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -86,11 +80,6 @@
         <fgColor rgb="004F46E5"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -104,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -131,8 +120,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -928,15 +915,15 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="30" customHeight="1">
+    <row r="37">
       <c r="B37" s="8" t="inlineStr">
         <is>
           <t>Update the status column on the Pages sheet after each page passes local QA. Live QA stays "Pending deploy" until boardexambd.com is live. The 404.html utility page is tracked on Pages but excluded from progress totals and the sitemap.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="20" customHeight="1"/>
-    <row r="39" ht="20" customHeight="1"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B37:G39"/>
@@ -1173,27 +1160,27 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>index, follow</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="O2" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>WebSite + Organization + WebPage</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -1208,12 +1195,12 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -1223,7 +1210,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -1231,16 +1218,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W2" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X2" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr">
         <is>
           <t>2026-11-15</t>
@@ -1301,47 +1284,47 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O3" s="11" t="inlineStr">
+        <is>
+          <t>CollectionPage + ItemList + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O3" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -1351,7 +1334,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -1359,16 +1342,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W3" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X3" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr">
         <is>
           <t>2026-11-15</t>
@@ -1429,47 +1408,47 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O4" s="11" t="inlineStr">
+        <is>
+          <t>CollectionPage + ItemList + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O4" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -1479,7 +1458,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -1487,16 +1466,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W4" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X4" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr">
         <is>
           <t>2026-11-15</t>
@@ -1504,7 +1479,7 @@
       </c>
       <c r="Z4" s="11" t="inlineStr">
         <is>
-          <t>Rebuilt hub with verified HSC dates, guide cards, timeline and FAQs.</t>
+          <t>Rebuilt hub with verified SSC dates, guide cards, timeline and FAQs.</t>
         </is>
       </c>
     </row>
@@ -1557,47 +1532,47 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O5" s="11" t="inlineStr">
+        <is>
+          <t>CollectionPage + ItemList + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O5" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -1607,7 +1582,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -1615,16 +1590,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W5" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X5" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr">
         <is>
           <t>2026-11-10</t>
@@ -1685,32 +1656,32 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>index, follow</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="O6" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>CollectionPage + ItemList + BreadcrumbList</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1720,12 +1691,12 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1735,7 +1706,7 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1743,16 +1714,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W6" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X6" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr">
         <is>
           <t>2026-11-15</t>
@@ -1813,57 +1780,57 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O7" s="11" t="inlineStr">
+        <is>
+          <t>Article + Organization + WebPage + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O7" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1871,16 +1838,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W7" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X7" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr">
         <is>
           <t>2026-11-15</t>
@@ -1941,57 +1904,57 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O8" s="11" t="inlineStr">
+        <is>
+          <t>Article + Organization + WebPage + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O8" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1999,16 +1962,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W8" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X8" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr">
         <is>
           <t>2026-11-15</t>
@@ -2069,57 +2028,57 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O9" s="11" t="inlineStr">
+        <is>
+          <t>Article + Organization + WebPage + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O9" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -2127,16 +2086,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W9" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X9" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr">
         <is>
           <t>2026-11-24</t>
@@ -2197,57 +2152,57 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O10" s="11" t="inlineStr">
+        <is>
+          <t>Article + Organization + WebPage + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O10" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -2255,16 +2210,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W10" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X10" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr">
         <is>
           <t>2026-11-15</t>
@@ -2325,57 +2276,57 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O11" s="11" t="inlineStr">
+        <is>
+          <t>Article + Organization + WebPage + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O11" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -2383,16 +2334,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W11" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X11" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr">
         <is>
           <t>2026-11-15</t>
@@ -2436,7 +2383,7 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>HSC and Alim result 2026 is scheduled for 29 October. Check your marksheet online at eboardresults.com or by SMS with this simple guide.</t>
+          <t>HSC and Alim result 2026 was published 31 October 2026 (pass rate 52.12%, 40,084 GPA-5). Check your marksheet online at eboardresults.com or by SMS with this simple guide.</t>
         </is>
       </c>
       <c r="H12">
@@ -2453,57 +2400,57 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O12" s="11" t="inlineStr">
+        <is>
+          <t>Article + Organization + WebPage + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O12" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
@@ -2511,24 +2458,20 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W12" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X12" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-11-07</t>
         </is>
       </c>
       <c r="Z12" s="11" t="inlineStr">
         <is>
-          <t>High priority: update on 29 October 2026 when result is published.</t>
+          <t>Result published 31 October 2026 (revised from 29 Oct); re-scrutiny window 1-7 Nov 2026.</t>
         </is>
       </c>
     </row>
@@ -2581,57 +2524,57 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O13" s="11" t="inlineStr">
+        <is>
+          <t>Article + Organization + WebPage + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O13" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
@@ -2639,16 +2582,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W13" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X13" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr"/>
       <c r="Y13" t="inlineStr">
         <is>
           <t>2026-12-15</t>
@@ -2709,57 +2648,57 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O14" s="11" t="inlineStr">
+        <is>
+          <t>Article + Organization + WebPage + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O14" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
@@ -2767,16 +2706,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W14" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X14" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr"/>
       <c r="Y14" t="inlineStr">
         <is>
           <t>2026-11-15</t>
@@ -2837,57 +2772,57 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O15" s="11" t="inlineStr">
+        <is>
+          <t>Article + Organization + WebPage + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O15" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
@@ -2895,16 +2830,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W15" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X15" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr">
         <is>
           <t>2026-11-20</t>
@@ -2965,57 +2896,57 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O16" s="11" t="inlineStr">
+        <is>
+          <t>Article + Organization + WebPage + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O16" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
@@ -3023,16 +2954,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W16" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X16" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr"/>
       <c r="Y16" t="inlineStr">
         <is>
           <t>2026-11-26</t>
@@ -3093,57 +3020,57 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O17" s="11" t="inlineStr">
+        <is>
+          <t>Article + Organization + WebPage + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O17" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
@@ -3151,16 +3078,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W17" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X17" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr"/>
       <c r="Y17" t="inlineStr">
         <is>
           <t>2026-11-15</t>
@@ -3221,57 +3144,57 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O18" s="11" t="inlineStr">
+        <is>
+          <t>Article + Organization + WebPage + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O18" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
@@ -3279,16 +3202,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W18" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X18" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr"/>
       <c r="Y18" t="inlineStr">
         <is>
           <t>2026-11-15</t>
@@ -3349,57 +3268,57 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O19" s="11" t="inlineStr">
+        <is>
+          <t>Article + Organization + WebPage + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O19" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
@@ -3407,16 +3326,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W19" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X19" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr"/>
       <c r="Y19" t="inlineStr">
         <is>
           <t>2026-11-15</t>
@@ -3424,7 +3339,7 @@
       </c>
       <c r="Z19" s="11" t="inlineStr">
         <is>
-          <t>Test tentative 4 Dec 2026; depends on HSC result 29 Oct.</t>
+          <t>Test tentative 4 Dec 2026; depends on HSC result published 31 Oct 2026.</t>
         </is>
       </c>
     </row>
@@ -3477,57 +3392,57 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O20" s="11" t="inlineStr">
+        <is>
+          <t>Article + Organization + WebPage + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O20" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
@@ -3535,16 +3450,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W20" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X20" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr"/>
       <c r="Y20" t="inlineStr">
         <is>
           <t>2026-11-13</t>
@@ -3605,57 +3516,57 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O21" s="11" t="inlineStr">
+        <is>
+          <t>Article + Organization + WebPage + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O21" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
@@ -3663,16 +3574,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W21" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X21" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr"/>
       <c r="Y21" t="inlineStr">
         <is>
           <t>2026-12-01</t>
@@ -3733,57 +3640,57 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>index, follow</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O22" s="11" t="inlineStr">
+        <is>
+          <t>Article + Organization + WebPage + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O22" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
@@ -3791,16 +3698,12 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W22" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X22" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr"/>
       <c r="Y22" t="inlineStr">
         <is>
           <t>2026-11-15</t>
@@ -3861,27 +3764,27 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>noindex, follow</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="O23" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>WebPage</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -3896,7 +3799,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -3911,7 +3814,7 @@
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
@@ -3919,16 +3822,13 @@
           <t>Pending deploy</t>
         </is>
       </c>
-      <c r="W23" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="X23" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr"/>
       <c r="Z23" s="11" t="inlineStr">
         <is>
           <t>noindex utility page.</t>
@@ -4341,7 +4241,7 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>HSC result is scheduled for 29 October 2026; page needs a post-result update.</t>
+          <t>HSC result was published on 31 October 2026 (revised from 29 Oct); page updated with pass rate, GPA-5 and SMS number.</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -4351,17 +4251,17 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>Update the result status, steps and FAQ on 29 October 2026.</t>
+          <t>Re-check the page after the 1-7 Nov 2026 re-scrutiny window closes.</t>
         </is>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-31</t>
         </is>
       </c>
     </row>
@@ -4841,12 +4741,12 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>SEO overhaul</t>
+          <t>HSC result published 31 October 2026; site-wide date refresh</t>
         </is>
       </c>
     </row>

</xml_diff>